<commit_message>
Replace hardcoded sensitive values in secrets with environment variable references for improved security
</commit_message>
<xml_diff>
--- a/Melpay LATEST.xlsx
+++ b/Melpay LATEST.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ike/Desktop/Project Destiny/replacement/melpay/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E17B835-08F6-7745-9777-8DECF8D1B984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{148709C7-5AF8-284F-9AEC-26B3226B9C7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3440" yWindow="500" windowWidth="30160" windowHeight="20500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TransactionHistory" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="9">
   <si>
     <t>type</t>
   </si>
@@ -59,6 +59,9 @@
   </si>
   <si>
     <t>FEBRUARY</t>
+  </si>
+  <si>
+    <t>great</t>
   </si>
 </sst>
 </file>
@@ -270,7 +273,7 @@
     </row>
     <row r="3" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B3">
         <v>2000</v>
@@ -304,7 +307,7 @@
     </row>
     <row r="5" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B5">
         <v>5477</v>

</xml_diff>

<commit_message>
Add authorization to the Home index and show actions
</commit_message>
<xml_diff>
--- a/Melpay LATEST.xlsx
+++ b/Melpay LATEST.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="8">
   <si>
     <t xml:space="preserve">type</t>
   </si>
@@ -37,13 +37,10 @@
     <t xml:space="preserve">phone number</t>
   </si>
   <si>
-    <t xml:space="preserve">orchard</t>
+    <t xml:space="preserve">flight</t>
   </si>
   <si>
     <t xml:space="preserve">Salary January</t>
-  </si>
-  <si>
-    <t xml:space="preserve">deposit</t>
   </si>
   <si>
     <t xml:space="preserve">FEBRUARY</t>
@@ -57,7 +54,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -79,6 +76,11 @@
       <name val="Arial"/>
       <family val="0"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -122,16 +124,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -261,124 +271,124 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="11.5078125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="7.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="7.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="0" t="n">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="n">
         <v>1000</v>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C2" s="2" t="n">
         <v>45413</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="0" t="n">
+      <c r="E2" s="1" t="n">
         <v>701450691</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="0" t="n">
+      <c r="A3" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1" t="n">
         <v>2000</v>
       </c>
-      <c r="C3" s="1" t="n">
+      <c r="C3" s="2" t="n">
         <v>45414</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="0" t="n">
+      <c r="E3" s="1" t="n">
         <v>701450692</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="0" t="n">
+      <c r="A4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="1" t="n">
         <v>5000</v>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" s="2" t="n">
         <v>45415</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="0" t="n">
+      <c r="E4" s="1" t="n">
         <v>701450693</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="0" t="n">
+      <c r="A5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1" t="n">
         <v>5477</v>
       </c>
-      <c r="C5" s="1" t="n">
+      <c r="C5" s="2" t="n">
         <v>45417</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="0" t="n">
+      <c r="E5" s="1" t="n">
         <v>701450694</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>4593</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>45422</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>701450695</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="0" t="n">
-        <v>4593</v>
-      </c>
-      <c r="C6" s="1" t="n">
-        <v>45422</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" s="0" t="n">
-        <v>701450695</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="0" t="n">
-        <v>6000</v>
-      </c>
-      <c r="D7" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="0" t="n">
+      <c r="E7" s="1" t="n">
         <v>734245034</v>
       </c>
     </row>

</xml_diff>